<commit_message>
tabtools: Add sparklines feature to table1_tc and expand QA suite
</commit_message>
<xml_diff>
--- a/tabtools/demo/regtab_mixed.xlsx
+++ b/tabtools/demo/regtab_mixed.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="210" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="280" uniqueCount="53">
   <si>
     <t>Table 3. Mixed Effects Model</t>
   </si>
@@ -178,10 +178,1302 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
-  <fonts count="922">
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
+  <fonts count="1229">
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
     </font>
     <font>
       <sz val="11"/>
@@ -4068,7 +5360,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="691">
+  <borders count="921">
     <border>
       <left/>
       <right/>
@@ -8816,11 +10108,1591 @@
       <bottom style="thin"/>
       <diagonal style="none"/>
     </border>
+    <border/>
+    <border/>
+    <border/>
+    <border/>
+    <border/>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="thin"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="thin"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="thin"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="thin"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="thin"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="thin"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="thin"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right style="none"/>
+      <top style="thin"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="thin"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="thin"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="thin"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="thin"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="thin"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="thin"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="thin"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="thin"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="691">
+  <cellXfs count="921">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0"/>
@@ -11534,6 +14406,911 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="921" fillId="0" borderId="690" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="691" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="692" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="693" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="694" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="695" xfId="0"/>
+    <xf numFmtId="0" fontId="922" fillId="0" borderId="696" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="923" fillId="0" borderId="697" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="924" fillId="0" borderId="698" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="925" fillId="0" borderId="699" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="926" fillId="0" borderId="700" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="927" fillId="0" borderId="701" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="929" fillId="0" borderId="702" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="931" fillId="0" borderId="703" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="933" fillId="0" borderId="704" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="934" fillId="0" borderId="705" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="935" fillId="0" borderId="706" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="936" fillId="0" borderId="707" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="937" fillId="0" borderId="708" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="938" fillId="0" borderId="709" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="939" fillId="0" borderId="710" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="940" fillId="0" borderId="711" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="941" fillId="0" borderId="712" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="942" fillId="0" borderId="713" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="943" fillId="0" borderId="714" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="944" fillId="0" borderId="715" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="945" fillId="0" borderId="716" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="946" fillId="0" borderId="717" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="947" fillId="0" borderId="718" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="948" fillId="0" borderId="719" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="949" fillId="0" borderId="720" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="950" fillId="0" borderId="721" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="951" fillId="0" borderId="722" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="952" fillId="0" borderId="723" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="953" fillId="0" borderId="724" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="954" fillId="0" borderId="725" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="955" fillId="0" borderId="726" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="956" fillId="0" borderId="727" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="957" fillId="0" borderId="728" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="958" fillId="0" borderId="729" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="959" fillId="0" borderId="730" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="961" fillId="0" borderId="731" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="963" fillId="0" borderId="732" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="965" fillId="0" borderId="733" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="967" fillId="0" borderId="734" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="969" fillId="0" borderId="735" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="970" fillId="0" borderId="736" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="971" fillId="0" borderId="737" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="972" fillId="0" borderId="738" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="973" fillId="0" borderId="739" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="974" fillId="0" borderId="740" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="975" fillId="0" borderId="741" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="976" fillId="0" borderId="742" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="977" fillId="0" borderId="743" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="978" fillId="0" borderId="744" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="979" fillId="0" borderId="745" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="980" fillId="0" borderId="746" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="981" fillId="0" borderId="747" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="982" fillId="0" borderId="748" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="984" fillId="0" borderId="749" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="986" fillId="0" borderId="750" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="988" fillId="0" borderId="751" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="990" fillId="0" borderId="752" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="991" fillId="0" borderId="753" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="992" fillId="0" borderId="754" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="993" fillId="0" borderId="755" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="994" fillId="0" borderId="756" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="995" fillId="0" borderId="757" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="996" fillId="0" borderId="758" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="997" fillId="0" borderId="759" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="998" fillId="0" borderId="760" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="999" fillId="0" borderId="761" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1000" fillId="0" borderId="762" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1001" fillId="0" borderId="763" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1002" fillId="0" borderId="764" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1003" fillId="0" borderId="765" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1004" fillId="0" borderId="766" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1005" fillId="0" borderId="767" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1006" fillId="0" borderId="768" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1007" fillId="0" borderId="769" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1008" fillId="0" borderId="770" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1009" fillId="0" borderId="771" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1010" fillId="0" borderId="772" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1011" fillId="0" borderId="773" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1012" fillId="0" borderId="774" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1013" fillId="0" borderId="775" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1014" fillId="0" borderId="776" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1015" fillId="0" borderId="777" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1016" fillId="0" borderId="778" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1017" fillId="0" borderId="779" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1018" fillId="0" borderId="780" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1019" fillId="0" borderId="781" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1020" fillId="0" borderId="782" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1021" fillId="0" borderId="783" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1022" fillId="0" borderId="784" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1023" fillId="0" borderId="785" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1024" fillId="0" borderId="786" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1025" fillId="0" borderId="787" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1026" fillId="0" borderId="788" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1027" fillId="0" borderId="789" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1028" fillId="0" borderId="790" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1029" fillId="0" borderId="791" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1030" fillId="0" borderId="792" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1031" fillId="0" borderId="793" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1032" fillId="0" borderId="794" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1033" fillId="0" borderId="795" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1034" fillId="0" borderId="796" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1035" fillId="0" borderId="797" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1036" fillId="0" borderId="798" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1037" fillId="0" borderId="799" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1038" fillId="0" borderId="800" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1039" fillId="0" borderId="801" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1040" fillId="0" borderId="802" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1041" fillId="0" borderId="803" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1042" fillId="0" borderId="804" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1043" fillId="0" borderId="805" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1044" fillId="0" borderId="806" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1045" fillId="0" borderId="807" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1046" fillId="0" borderId="808" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1047" fillId="0" borderId="809" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1048" fillId="0" borderId="810" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1049" fillId="0" borderId="811" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1050" fillId="0" borderId="812" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1051" fillId="0" borderId="813" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1052" fillId="0" borderId="814" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1053" fillId="0" borderId="815" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1054" fillId="0" borderId="816" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1055" fillId="0" borderId="817" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1056" fillId="0" borderId="818" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1057" fillId="0" borderId="819" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1058" fillId="0" borderId="820" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1059" fillId="0" borderId="821" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1060" fillId="0" borderId="822" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1061" fillId="0" borderId="823" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1062" fillId="0" borderId="824" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1063" fillId="0" borderId="825" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1064" fillId="0" borderId="826" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1065" fillId="0" borderId="827" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1066" fillId="0" borderId="828" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1067" fillId="0" borderId="829" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1068" fillId="0" borderId="830" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1069" fillId="0" borderId="831" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1070" fillId="0" borderId="832" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1071" fillId="0" borderId="833" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1072" fillId="0" borderId="834" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1073" fillId="0" borderId="835" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1074" fillId="0" borderId="836" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1075" fillId="0" borderId="837" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1076" fillId="0" borderId="838" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1077" fillId="0" borderId="839" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1078" fillId="0" borderId="840" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1079" fillId="0" borderId="841" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1080" fillId="0" borderId="842" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1081" fillId="0" borderId="843" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1082" fillId="0" borderId="844" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1083" fillId="0" borderId="845" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1084" fillId="0" borderId="846" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1085" fillId="0" borderId="847" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1086" fillId="0" borderId="848" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1087" fillId="0" borderId="849" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1088" fillId="0" borderId="850" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1090" fillId="0" borderId="851" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1092" fillId="0" borderId="852" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1094" fillId="0" borderId="853" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1096" fillId="0" borderId="854" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1098" fillId="0" borderId="855" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1100" fillId="0" borderId="856" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1102" fillId="0" borderId="857" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1104" fillId="0" borderId="858" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1106" fillId="0" borderId="859" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1108" fillId="0" borderId="860" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1110" fillId="0" borderId="861" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1112" fillId="0" borderId="862" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1114" fillId="0" borderId="863" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1116" fillId="0" borderId="864" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1118" fillId="0" borderId="865" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1120" fillId="0" borderId="866" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1122" fillId="0" borderId="867" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1124" fillId="0" borderId="868" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1126" fillId="0" borderId="869" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1128" fillId="0" borderId="870" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1130" fillId="0" borderId="871" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1132" fillId="0" borderId="872" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1134" fillId="0" borderId="873" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1136" fillId="0" borderId="874" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1138" fillId="0" borderId="875" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1140" fillId="0" borderId="876" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1142" fillId="0" borderId="877" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1144" fillId="0" borderId="878" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1146" fillId="0" borderId="879" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1148" fillId="0" borderId="880" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1150" fillId="0" borderId="881" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1152" fillId="0" borderId="882" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1154" fillId="0" borderId="883" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1156" fillId="0" borderId="884" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1158" fillId="0" borderId="885" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1160" fillId="0" borderId="886" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1162" fillId="0" borderId="887" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1164" fillId="0" borderId="888" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1166" fillId="0" borderId="889" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1168" fillId="0" borderId="890" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1170" fillId="0" borderId="891" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1172" fillId="0" borderId="892" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1174" fillId="0" borderId="893" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1176" fillId="0" borderId="894" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1178" fillId="0" borderId="895" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1180" fillId="0" borderId="896" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1182" fillId="0" borderId="897" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1184" fillId="0" borderId="898" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1186" fillId="0" borderId="899" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1188" fillId="0" borderId="900" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1190" fillId="0" borderId="901" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1192" fillId="0" borderId="902" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1194" fillId="0" borderId="903" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1196" fillId="0" borderId="904" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1198" fillId="0" borderId="905" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1200" fillId="0" borderId="906" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1202" fillId="0" borderId="907" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1204" fillId="0" borderId="908" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1206" fillId="0" borderId="909" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1208" fillId="0" borderId="910" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1210" fillId="0" borderId="911" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1212" fillId="0" borderId="912" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1214" fillId="0" borderId="913" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1216" fillId="0" borderId="914" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1218" fillId="0" borderId="915" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1220" fillId="0" borderId="916" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1222" fillId="0" borderId="917" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1224" fillId="0" borderId="918" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1226" fillId="0" borderId="919" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1228" fillId="0" borderId="920" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -11549,247 +15326,247 @@
   <dimension ref="A1:E14"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="19.7109375" style="462" customWidth="true"/>
-    <col min="3" max="3" width="5.11328125" style="463" customWidth="true"/>
-    <col min="4" max="4" width="11.11328125" style="464" customWidth="true"/>
-    <col min="5" max="5" width="7.7109375" style="465" customWidth="true"/>
+    <col min="2" max="2" width="19.7109375" style="692" customWidth="true"/>
+    <col min="3" max="3" width="5.11328125" style="693" customWidth="true"/>
+    <col min="4" max="4" width="11.11328125" style="694" customWidth="true"/>
+    <col min="5" max="5" width="7.7109375" style="695" customWidth="true"/>
   </cols>
   <sheetData>
-    <row r="1" s="461" customFormat="true" ht="30" customHeight="true">
-      <c r="A1" s="621" t="s">
+    <row r="1" s="691" customFormat="true" ht="30" customHeight="true">
+      <c r="A1" s="851" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="622" t="s">
+      <c r="B1" s="852" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="623" t="s">
+      <c r="C1" s="853" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="624" t="s">
+      <c r="D1" s="854" t="s">
         <v>1</v>
       </c>
-      <c r="E1" s="625" t="s">
+      <c r="E1" s="855" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="626" t="s">
+      <c r="A2" s="856" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="627" t="s">
+      <c r="B2" s="857" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="628" t="s">
+      <c r="C2" s="858" t="s">
         <v>1</v>
       </c>
-      <c r="D2" s="629" t="s">
+      <c r="D2" s="859" t="s">
         <v>1</v>
       </c>
-      <c r="E2" s="630" t="s">
+      <c r="E2" s="860" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="631" t="s">
+      <c r="A3" s="861" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="632" t="s">
+      <c r="B3" s="862" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="633" t="s">
+      <c r="C3" s="863" t="s">
         <v>13</v>
       </c>
-      <c r="D3" s="634" t="s">
+      <c r="D3" s="864" t="s">
         <v>25</v>
       </c>
-      <c r="E3" s="635" t="s">
+      <c r="E3" s="865" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="636" t="s">
+      <c r="A4" s="866" t="s">
         <v>1</v>
       </c>
-      <c r="B4" s="637" t="s">
+      <c r="B4" s="867" t="s">
         <v>2</v>
       </c>
-      <c r="C4" s="638" t="s">
+      <c r="C4" s="868" t="s">
         <v>35</v>
       </c>
-      <c r="D4" s="639" t="s">
+      <c r="D4" s="869" t="s">
         <v>26</v>
       </c>
-      <c r="E4" s="640" t="s">
+      <c r="E4" s="870" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="641" t="s">
+      <c r="A5" s="871" t="s">
         <v>1</v>
       </c>
-      <c r="B5" s="642" t="s">
+      <c r="B5" s="872" t="s">
         <v>3</v>
       </c>
-      <c r="C5" s="643" t="s">
+      <c r="C5" s="873" t="s">
         <v>36</v>
       </c>
-      <c r="D5" s="644" t="s">
+      <c r="D5" s="874" t="s">
         <v>46</v>
       </c>
-      <c r="E5" s="645" t="s">
+      <c r="E5" s="875" t="s">
         <v>51</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="646" t="s">
+      <c r="A6" s="876" t="s">
         <v>1</v>
       </c>
-      <c r="B6" s="647" t="s">
+      <c r="B6" s="877" t="s">
         <v>4</v>
       </c>
-      <c r="C6" s="648" t="s">
+      <c r="C6" s="878" t="s">
         <v>37</v>
       </c>
-      <c r="D6" s="649" t="s">
+      <c r="D6" s="879" t="s">
         <v>47</v>
       </c>
-      <c r="E6" s="650" t="s">
+      <c r="E6" s="880" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="651" t="s">
+      <c r="A7" s="881" t="s">
         <v>1</v>
       </c>
-      <c r="B7" s="652" t="s">
+      <c r="B7" s="882" t="s">
         <v>5</v>
       </c>
-      <c r="C7" s="653" t="s">
+      <c r="C7" s="883" t="s">
         <v>38</v>
       </c>
-      <c r="D7" s="654" t="s">
+      <c r="D7" s="884" t="s">
         <v>48</v>
       </c>
-      <c r="E7" s="655" t="s">
+      <c r="E7" s="885" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="656" t="s">
+      <c r="A8" s="886" t="s">
         <v>1</v>
       </c>
-      <c r="B8" s="657" t="s">
+      <c r="B8" s="887" t="s">
         <v>6</v>
       </c>
-      <c r="C8" s="658" t="s">
+      <c r="C8" s="888" t="s">
         <v>39</v>
       </c>
-      <c r="D8" s="659" t="s">
+      <c r="D8" s="889" t="s">
         <v>49</v>
       </c>
-      <c r="E8" s="660" t="s">
+      <c r="E8" s="890" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="661" t="s">
+      <c r="A9" s="891" t="s">
         <v>1</v>
       </c>
-      <c r="B9" s="662" t="s">
+      <c r="B9" s="892" t="s">
         <v>7</v>
       </c>
-      <c r="C9" s="663" t="s">
+      <c r="C9" s="893" t="s">
         <v>40</v>
       </c>
-      <c r="D9" s="664" t="s">
+      <c r="D9" s="894" t="s">
         <v>50</v>
       </c>
-      <c r="E9" s="665" t="s">
+      <c r="E9" s="895" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="666" t="s">
+      <c r="A10" s="896" t="s">
         <v>1</v>
       </c>
-      <c r="B10" s="667" t="s">
+      <c r="B10" s="897" t="s">
         <v>8</v>
       </c>
-      <c r="C10" s="668" t="s">
+      <c r="C10" s="898" t="s">
         <v>41</v>
       </c>
-      <c r="D10" s="669" t="s">
+      <c r="D10" s="899" t="s">
         <v>1</v>
       </c>
-      <c r="E10" s="670" t="s">
+      <c r="E10" s="900" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="671" t="s">
+      <c r="A11" s="901" t="s">
         <v>1</v>
       </c>
-      <c r="B11" s="672" t="s">
+      <c r="B11" s="902" t="s">
         <v>9</v>
       </c>
-      <c r="C11" s="673" t="s">
+      <c r="C11" s="903" t="s">
         <v>42</v>
       </c>
-      <c r="D11" s="674" t="s">
+      <c r="D11" s="904" t="s">
         <v>1</v>
       </c>
-      <c r="E11" s="675" t="s">
+      <c r="E11" s="905" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="676" t="s">
+      <c r="A12" s="906" t="s">
         <v>1</v>
       </c>
-      <c r="B12" s="677" t="s">
+      <c r="B12" s="907" t="s">
         <v>10</v>
       </c>
-      <c r="C12" s="678" t="s">
+      <c r="C12" s="908" t="s">
         <v>43</v>
       </c>
-      <c r="D12" s="679" t="s">
+      <c r="D12" s="909" t="s">
         <v>1</v>
       </c>
-      <c r="E12" s="680" t="s">
+      <c r="E12" s="910" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="681" t="s">
+      <c r="A13" s="911" t="s">
         <v>1</v>
       </c>
-      <c r="B13" s="682" t="s">
+      <c r="B13" s="912" t="s">
         <v>11</v>
       </c>
-      <c r="C13" s="683" t="s">
+      <c r="C13" s="913" t="s">
         <v>44</v>
       </c>
-      <c r="D13" s="684" t="s">
+      <c r="D13" s="914" t="s">
         <v>1</v>
       </c>
-      <c r="E13" s="685" t="s">
+      <c r="E13" s="915" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="686" t="s">
+      <c r="A14" s="916" t="s">
         <v>1</v>
       </c>
-      <c r="B14" s="687" t="s">
+      <c r="B14" s="917" t="s">
         <v>12</v>
       </c>
-      <c r="C14" s="688" t="s">
+      <c r="C14" s="918" t="s">
         <v>52</v>
       </c>
-      <c r="D14" s="689" t="s">
+      <c r="D14" s="919" t="s">
         <v>1</v>
       </c>
-      <c r="E14" s="690" t="s">
+      <c r="E14" s="920" t="s">
         <v>1</v>
       </c>
     </row>

</xml_diff>